<commit_message>
Finalize Q10437 business task and Windows package
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R52b914c6355d4318"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R7a699baf18c14ef6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -440,122 +440,114 @@
     </x:row>
     <x:row r="5" ht="33" customHeight="1">
       <x:c r="A5" s="16" t="str">
-        <x:v>业务角色</x:v>
+        <x:v>输入来源</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>广告数据平台发布工程师</x:v>
+        <x:v>脱敏分片清单、失败处置策略、发布参数、Chart值文件和模板骨架</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="33" customHeight="1">
       <x:c r="A6" s="16" t="str">
-        <x:v>结果消费者</x:v>
+        <x:v>输入获取方式</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
-        <x:v>日报值班负责人和广告平台维护者</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="33" customHeight="1">
+        <x:v>解压输入数据包后读取input_data下的starter与tools</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="16" t="str">
-        <x:v>输入来源</x:v>
+        <x:v>原始输入文件</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
-        <x:v>脱敏分片清单、失败处置策略、发布参数、Chart值文件和模板骨架</x:v>
+        <x:v>shard_inputs.csv；failure_plan.json；release_profile.json；values.yaml；Chart.yaml；resources.yaml</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="33" customHeight="1">
       <x:c r="A8" s="16" t="str">
-        <x:v>输入获取方式</x:v>
+        <x:v>目标输出文件</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>解压输入数据包后读取input_data下的starter与tools</x:v>
+        <x:v>完成Chart；渲染对象；分片Job登记；重试决策；聚合契约；Helm检查记录；发布审查</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="16" t="str">
-        <x:v>原始输入文件</x:v>
+        <x:v>核心操作链</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>shard_inputs.csv；failure_plan.json；release_profile.json；values.yaml；Chart.yaml；resources.yaml</x:v>
+        <x:v>关联输入；生成首次Job；生成有限重试和隔离；形成协调与聚合契约；执行Helm检查与渲染；整理报告并回查</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="33" customHeight="1">
       <x:c r="A10" s="16" t="str">
-        <x:v>目标输出文件</x:v>
+        <x:v>业务角色与消费者</x:v>
       </x:c>
       <x:c r="B10" s="17" t="str">
-        <x:v>完成Chart；渲染对象；分片Job登记；重试决策；聚合契约；Helm检查记录；发布审查</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="48" customHeight="1">
+        <x:v>广告数据平台发布工程师完成设计，日报值班负责人和广告平台维护者使用发布材料</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="33" customHeight="1">
       <x:c r="A11" s="16" t="str">
-        <x:v>核心操作链</x:v>
+        <x:v>分片映射规则</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>关联输入；生成首次Job；生成有限重试和隔离；形成协调与聚合契约；执行Helm检查与渲染；整理报告并回查</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="33" customHeight="1">
+        <x:v>每个分片生成一个首次Job，映射序号使用分片清单的零起始物理顺序</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="16" t="str">
-        <x:v>分片映射规则</x:v>
+        <x:v>失败处置规则</x:v>
       </x:c>
       <x:c r="B12" s="17" t="str">
-        <x:v>每个分片生成一个首次Job，映射序号使用分片清单的零起始物理顺序</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="48" customHeight="1">
+        <x:v>只有rerun_planned为true的故障生成一次第二次Job；quarantined终态进入隔离且不参与聚合</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="33" customHeight="1">
       <x:c r="A13" s="16" t="str">
-        <x:v>失败处置规则</x:v>
+        <x:v>聚合规则</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>只有rerun_planned为true的故障生成一次第二次Job；quarantined终态进入隔离且不参与聚合</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="33" customHeight="1">
+        <x:v>等待全部分片终态，只纳入最终成功分片一次，处理量从当前分片清单逐项求和</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="16" t="str">
-        <x:v>聚合规则</x:v>
+        <x:v>协调规则</x:v>
       </x:c>
       <x:c r="B14" s="17" t="str">
-        <x:v>等待全部分片终态，只纳入最终成功分片一次，处理量从当前分片清单逐项求和</x:v>
+        <x:v>Lease与聚合Job使用release_profile.json中的同一锁标识，Lease时长也取自该文件</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="16" t="str">
-        <x:v>协调规则</x:v>
+        <x:v>Helm规则</x:v>
       </x:c>
       <x:c r="B15" s="17" t="str">
-        <x:v>Lease与聚合Job使用release_profile.json中的同一锁标识，Lease时长也取自该文件</x:v>
+        <x:v>必须使用Files.Get、模板循环、Values、Release上下文、lint --strict和template</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="16" t="str">
-        <x:v>Helm规则</x:v>
+        <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B16" s="17" t="str">
-        <x:v>必须使用Files.Get、模板循环、Values、Release上下文、lint --strict和template</x:v>
+        <x:v>npm run build-release正常结束，完成Chart、渲染对象和五份报告可读且关系闭合</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="16" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>可验证点</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
-        <x:v>npm run build-release正常结束，完成Chart、渲染对象和五份报告可读且关系闭合</x:v>
+        <x:v>分片与首次Job一一对应；重试与隔离只受failure_plan.json控制；聚合集合和处理量可从当前输入复算；Lease与聚合Job的协调字段一致；报告与Helm渲染对象关系闭合</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="33" customHeight="1">
-      <x:c r="A18" s="16" t="str">
-        <x:v>错误收口</x:v>
-      </x:c>
-      <x:c r="B18" s="17" t="str">
-        <x:v>输入缺失、关系矛盾、模板未完成或Helm检查失败时返回非零状态且不保留output</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="33" customHeight="1">
-      <x:c r="A19" s="18" t="str">
+      <x:c r="A18" s="18" t="str">
         <x:v>不适合作为评分点的内容</x:v>
       </x:c>
-      <x:c r="B19" s="19" t="str">
-        <x:v>辅助函数拆分、等价资源命名、无业务顺序的报告行序和等义错误文案</x:v>
+      <x:c r="B18" s="19" t="str">
+        <x:v>辅助函数拆分、等价资源命名、无业务顺序的报告行序和等义问题文案</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>